<commit_message>
update- debug (in work)
</commit_message>
<xml_diff>
--- a/user_inputs/plot_terms.xlsx
+++ b/user_inputs/plot_terms.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="61">
   <si>
     <t>Plot?</t>
   </si>
@@ -88,9 +88,6 @@
     <t>LVDT-2 Status - Calibration</t>
   </si>
   <si>
-    <t>Calibration Workbook Sheets - Attachment Index</t>
-  </si>
-  <si>
     <t>SN</t>
   </si>
   <si>
@@ -133,9 +130,6 @@
     <t>LVDT-2 Status</t>
   </si>
   <si>
-    <t>Calibration Workbook Sheets</t>
-  </si>
-  <si>
     <t>Document Profile</t>
   </si>
   <si>
@@ -151,16 +145,10 @@
     <t>Calibration</t>
   </si>
   <si>
-    <t>Attachment Index</t>
-  </si>
-  <si>
     <t>psia</t>
   </si>
   <si>
     <t>ω</t>
-  </si>
-  <si>
-    <t>sheets</t>
   </si>
   <si>
     <t>4.0</t>
@@ -566,16 +554,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K15"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
-    <col min="2" max="2" width="48.7109375" customWidth="1"/>
+    <col min="2" max="2" width="47.7109375" customWidth="1"/>
     <col min="3" max="4" width="12.7109375" customWidth="1"/>
-    <col min="5" max="5" width="29.7109375" customWidth="1"/>
+    <col min="5" max="5" width="26.7109375" customWidth="1"/>
     <col min="6" max="6" width="23.7109375" customWidth="1"/>
     <col min="7" max="10" width="12.7109375" customWidth="1"/>
-    <col min="11" max="11" width="48.7109375" customWidth="1"/>
+    <col min="11" max="11" width="47.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11">
@@ -618,13 +606,13 @@
         <v>11</v>
       </c>
       <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
         <v>25</v>
       </c>
-      <c r="E2" t="s">
-        <v>26</v>
-      </c>
       <c r="F2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K2" t="s">
         <v>11</v>
@@ -635,13 +623,13 @@
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F3" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K3" t="s">
         <v>12</v>
@@ -652,19 +640,19 @@
         <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="H4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I4" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="K4" t="s">
         <v>13</v>
@@ -675,13 +663,13 @@
         <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="K5" t="s">
         <v>14</v>
@@ -692,25 +680,25 @@
         <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G6" t="s">
+        <v>43</v>
+      </c>
+      <c r="H6" t="s">
         <v>46</v>
       </c>
-      <c r="H6" t="s">
-        <v>50</v>
-      </c>
       <c r="I6" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="J6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="K6" t="s">
         <v>15</v>
@@ -721,25 +709,25 @@
         <v>16</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G7" t="s">
+        <v>44</v>
+      </c>
+      <c r="H7" t="s">
         <v>47</v>
       </c>
-      <c r="H7" t="s">
-        <v>51</v>
-      </c>
       <c r="I7" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="J7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="K7" t="s">
         <v>16</v>
@@ -750,19 +738,19 @@
         <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H8" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="I8" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="K8" t="s">
         <v>17</v>
@@ -773,19 +761,19 @@
         <v>18</v>
       </c>
       <c r="D9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I9" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="K9" t="s">
         <v>18</v>
@@ -796,19 +784,19 @@
         <v>19</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F10" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H10" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="I10" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="K10" t="s">
         <v>19</v>
@@ -819,19 +807,19 @@
         <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F11" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H11" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I11" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="K11" t="s">
         <v>20</v>
@@ -842,19 +830,19 @@
         <v>21</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F12" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="H12" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="I12" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="K12" t="s">
         <v>21</v>
@@ -865,19 +853,19 @@
         <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F13" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H13" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="I13" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="K13" t="s">
         <v>22</v>
@@ -888,59 +876,30 @@
         <v>23</v>
       </c>
       <c r="D14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E14" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F14" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="H14" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="I14" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="K14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
-      <c r="B15" t="s">
-        <v>24</v>
-      </c>
-      <c r="D15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E15" t="s">
-        <v>39</v>
-      </c>
-      <c r="F15" t="s">
-        <v>45</v>
-      </c>
-      <c r="G15" t="s">
-        <v>48</v>
-      </c>
-      <c r="H15" t="s">
-        <v>49</v>
-      </c>
-      <c r="I15" t="s">
-        <v>49</v>
-      </c>
-      <c r="J15" t="s">
-        <v>48</v>
-      </c>
-      <c r="K15" t="s">
-        <v>24</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A16">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A15">
       <formula1>",Y,N"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D16">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D15">
       <formula1>"SN,Program,Space Vehicle"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
update - master spreadsheet sync
</commit_message>
<xml_diff>
--- a/user_inputs/plot_terms.xlsx
+++ b/user_inputs/plot_terms.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="74">
   <si>
     <t>Plot?</t>
   </si>
@@ -109,9 +109,6 @@
     <t>LVDT-2 Status - Calibration</t>
   </si>
   <si>
-    <t>LVDT-2 Pre-Trim - Calibration</t>
-  </si>
-  <si>
     <t>LVDT-2 Post-Trim - Calibration</t>
   </si>
   <si>
@@ -176,9 +173,6 @@
   </si>
   <si>
     <t>LVDT-2 Status</t>
-  </si>
-  <si>
-    <t>LVDT-2 Pre-Trim</t>
   </si>
   <si>
     <t>LVDT-2 Post-Trim</t>
@@ -599,7 +593,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
@@ -651,13 +645,13 @@
         <v>11</v>
       </c>
       <c r="D2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
         <v>33</v>
       </c>
-      <c r="E2" t="s">
-        <v>34</v>
-      </c>
       <c r="F2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="K2" t="s">
         <v>11</v>
@@ -668,13 +662,13 @@
         <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="K3" t="s">
         <v>12</v>
@@ -685,13 +679,13 @@
         <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F4" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="K4" t="s">
         <v>13</v>
@@ -702,13 +696,13 @@
         <v>14</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F5" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="K5" t="s">
         <v>14</v>
@@ -719,25 +713,25 @@
         <v>15</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H6" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="I6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J6" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="K6" t="s">
         <v>15</v>
@@ -748,13 +742,13 @@
         <v>16</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K7" t="s">
         <v>16</v>
@@ -765,25 +759,25 @@
         <v>17</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="G8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="H8" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="J8" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="K8" t="s">
         <v>17</v>
@@ -794,13 +788,13 @@
         <v>18</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K9" t="s">
         <v>18</v>
@@ -811,19 +805,19 @@
         <v>19</v>
       </c>
       <c r="D10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H10" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I10" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="K10" t="s">
         <v>19</v>
@@ -834,19 +828,19 @@
         <v>20</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H11" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="I11" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="K11" t="s">
         <v>20</v>
@@ -857,16 +851,16 @@
         <v>21</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F12" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="I12" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="K12" t="s">
         <v>21</v>
@@ -877,19 +871,19 @@
         <v>22</v>
       </c>
       <c r="D13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H13" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="I13" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K13" t="s">
         <v>22</v>
@@ -900,13 +894,13 @@
         <v>23</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F14" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="K14" t="s">
         <v>23</v>
@@ -917,13 +911,13 @@
         <v>24</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F15" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="K15" t="s">
         <v>24</v>
@@ -934,13 +928,13 @@
         <v>25</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F16" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="K16" t="s">
         <v>25</v>
@@ -951,13 +945,13 @@
         <v>26</v>
       </c>
       <c r="D17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F17" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K17" t="s">
         <v>26</v>
@@ -968,13 +962,13 @@
         <v>27</v>
       </c>
       <c r="D18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F18" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="K18" t="s">
         <v>27</v>
@@ -985,25 +979,25 @@
         <v>28</v>
       </c>
       <c r="D19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F19" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G19" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="H19" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="I19" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="J19" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="K19" t="s">
         <v>28</v>
@@ -1014,25 +1008,25 @@
         <v>29</v>
       </c>
       <c r="D20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F20" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="I20" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="J20" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="K20" t="s">
         <v>29</v>
@@ -1043,13 +1037,13 @@
         <v>30</v>
       </c>
       <c r="D21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F21" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K21" t="s">
         <v>30</v>
@@ -1060,41 +1054,24 @@
         <v>31</v>
       </c>
       <c r="D22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F22" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K22" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="23" spans="2:11">
-      <c r="B23" t="s">
-        <v>32</v>
-      </c>
-      <c r="D23" t="s">
-        <v>33</v>
-      </c>
-      <c r="E23" t="s">
-        <v>55</v>
-      </c>
-      <c r="F23" t="s">
-        <v>60</v>
-      </c>
-      <c r="K23" t="s">
-        <v>32</v>
-      </c>
-    </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A24">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A23">
       <formula1>",Y,N"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D24">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D23">
       <formula1>"SN,Program,Space Vehicle"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>